<commit_message>
TeacherTimeTable.py added constrain v1
</commit_message>
<xml_diff>
--- a/teacher_timetable_data.xlsx
+++ b/teacher_timetable_data.xlsx
@@ -9,7 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="Teachers" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Classes" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Subjects" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Students" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="45">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -57,37 +57,34 @@
     <t xml:space="preserve">BCA_A</t>
   </si>
   <si>
-    <t xml:space="preserve">CPP</t>
+    <t xml:space="preserve">MYSQL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_LAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Networks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OS</t>
   </si>
   <si>
     <t xml:space="preserve">BCA_B</t>
   </si>
   <si>
-    <t xml:space="preserve">JAVA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bsc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Python</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MYSQL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Java_LAB</t>
-  </si>
-  <si>
     <t xml:space="preserve">MYSQL_LAB</t>
   </si>
   <si>
-    <t xml:space="preserve">C_LAB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPP_LAB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Python_LAB</t>
+    <t xml:space="preserve">Web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DataMining</t>
   </si>
   <si>
     <t xml:space="preserve">Student_1</t>
@@ -241,7 +238,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -251,11 +248,11 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -264,6 +261,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -399,47 +400,47 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B2" s="3" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="3" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" s="3" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="3" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" s="3" t="n">
         <v>5</v>
       </c>
     </row>
@@ -477,147 +478,147 @@
       <c r="C1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="3" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="5" t="n">
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="3" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="5" t="n">
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="3" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4" t="s">
+      <c r="B11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -641,131 +642,131 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="6" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>22</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>32</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>38</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
student timetable in progress
</commit_message>
<xml_diff>
--- a/teacher_timetable_data.xlsx
+++ b/teacher_timetable_data.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="47">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -69,16 +69,22 @@
     <t xml:space="preserve">Networks</t>
   </si>
   <si>
+    <t xml:space="preserve">Bsc</t>
+  </si>
+  <si>
     <t xml:space="preserve">DS</t>
   </si>
   <si>
     <t xml:space="preserve">OS</t>
   </si>
   <si>
+    <t xml:space="preserve">Bcom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MYSQL_LAB</t>
+  </si>
+  <si>
     <t xml:space="preserve">BCA_B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MYSQL_LAB</t>
   </si>
   <si>
     <t xml:space="preserve">Web</t>
@@ -546,7 +552,7 @@
         <v>14</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>2</v>
@@ -557,7 +563,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>10</v>
@@ -571,10 +577,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>2</v>
@@ -585,10 +591,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>3</v>
@@ -599,10 +605,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>3</v>
@@ -613,10 +619,10 @@
         <v>4</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>17</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>2</v>
@@ -651,122 +657,122 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>